<commit_message>
sua loi thieu dinh nghia QUANTITATIVE_THRESHOLD
</commit_message>
<xml_diff>
--- a/coefficient.xlsx
+++ b/coefficient.xlsx
@@ -133,7 +133,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:N20"/>
-  <sheetFormatPr defaultColWidth="8.7578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.76953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -345,17 +345,17 @@
       <c r="N9" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E11" s="3" t="n">
-        <v>20</v>
+      <c r="B11" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="D11" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="E11" s="0" t="n">
+        <v>99</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>20</v>
@@ -365,17 +365,17 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>20</v>
+      <c r="B12" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="D12" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="E12" s="0" t="n">
+        <v>99</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>20</v>
@@ -385,17 +385,17 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E13" s="3" t="n">
-        <v>20</v>
+      <c r="B13" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="C13" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="D13" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="E13" s="0" t="n">
+        <v>99</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>20</v>
@@ -405,17 +405,17 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>20</v>
+      <c r="B14" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="C14" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="D14" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="E14" s="0" t="n">
+        <v>99</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>20</v>

</xml_diff>